<commit_message>
feat: add popularity scores
</commit_message>
<xml_diff>
--- a/input.xlsx
+++ b/input.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\anant\OneDrive\Documents\MSO Project\Sports_Scheduling_Project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D30675B5-2261-4538-90A5-9E408BD564DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6060F3D-A07F-4C5A-9426-6510AC5BD35A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{ABCAAF75-74DD-435C-8190-A0B94A49E869}"/>
   </bookViews>
@@ -65,9 +65,6 @@
     <t>Group</t>
   </si>
   <si>
-    <t>IsPopular</t>
-  </si>
-  <si>
     <t>IsStrong</t>
   </si>
   <si>
@@ -83,9 +80,6 @@
     <t>T1</t>
   </si>
   <si>
-    <t>Team 1</t>
-  </si>
-  <si>
     <t>North</t>
   </si>
   <si>
@@ -95,49 +89,55 @@
     <t>T2</t>
   </si>
   <si>
-    <t>Team 2</t>
-  </si>
-  <si>
     <t>T3</t>
   </si>
   <si>
-    <t>Team 3</t>
-  </si>
-  <si>
     <t>Center</t>
   </si>
   <si>
     <t>T4</t>
   </si>
   <si>
-    <t>Team 4</t>
-  </si>
-  <si>
     <t>T5</t>
   </si>
   <si>
-    <t>Team 5</t>
-  </si>
-  <si>
     <t>T6</t>
   </si>
   <si>
-    <t>Team 6</t>
-  </si>
-  <si>
     <t>T7</t>
   </si>
   <si>
-    <t>Team 7</t>
-  </si>
-  <si>
     <t>South</t>
   </si>
   <si>
     <t>T8</t>
   </si>
   <si>
-    <t>team 8</t>
+    <t>PopularityScore</t>
+  </si>
+  <si>
+    <t>Colo Colo</t>
+  </si>
+  <si>
+    <t>Universidad de Chile</t>
+  </si>
+  <si>
+    <t>Universidad Catolica</t>
+  </si>
+  <si>
+    <t>Cobreloa</t>
+  </si>
+  <si>
+    <t>Everton</t>
+  </si>
+  <si>
+    <t>La Serena</t>
+  </si>
+  <si>
+    <t>Universidad de Concepcion</t>
+  </si>
+  <si>
+    <t>Huachipato</t>
   </si>
 </sst>
 </file>
@@ -173,9 +173,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -226,13 +225,23 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{D4E3ACDC-C4F0-4E29-8A8A-C028DC907D21}" name="teams" displayName="teams" ref="A1:I9" tableType="queryTable" totalsRowShown="0">
-  <autoFilter ref="A1:I9" xr:uid="{D4E3ACDC-C4F0-4E29-8A8A-C028DC907D21}"/>
+  <autoFilter ref="A1:I9" xr:uid="{D4E3ACDC-C4F0-4E29-8A8A-C028DC907D21}">
+    <filterColumn colId="0" hiddenButton="1"/>
+    <filterColumn colId="1" hiddenButton="1"/>
+    <filterColumn colId="2" hiddenButton="1"/>
+    <filterColumn colId="3" hiddenButton="1"/>
+    <filterColumn colId="4" hiddenButton="1"/>
+    <filterColumn colId="5" hiddenButton="1"/>
+    <filterColumn colId="6" hiddenButton="1"/>
+    <filterColumn colId="7" hiddenButton="1"/>
+    <filterColumn colId="8" hiddenButton="1"/>
+  </autoFilter>
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{5BFF664F-09B1-4235-AF77-3F29199848BA}" uniqueName="1" name="TeamID" queryTableFieldId="1" dataDxfId="3"/>
     <tableColumn id="2" xr3:uid="{8AE8B0BE-87E9-4426-A8FD-93CCBB30D38D}" uniqueName="2" name="TeamName" queryTableFieldId="2" dataDxfId="2"/>
     <tableColumn id="3" xr3:uid="{D0BE88B4-B92B-4D1A-9034-C68DDE7496C1}" uniqueName="3" name="Region" queryTableFieldId="3" dataDxfId="1"/>
     <tableColumn id="4" xr3:uid="{F0A42F81-B903-4D5B-A92F-80C4EF9FD3B4}" uniqueName="4" name="Group" queryTableFieldId="4"/>
-    <tableColumn id="5" xr3:uid="{B8DC75BD-37EA-4DBA-BF62-3D46BDB6E93F}" uniqueName="5" name="IsPopular" queryTableFieldId="5"/>
+    <tableColumn id="5" xr3:uid="{B8DC75BD-37EA-4DBA-BF62-3D46BDB6E93F}" uniqueName="5" name="PopularityScore" queryTableFieldId="5"/>
     <tableColumn id="6" xr3:uid="{000CA2A6-8E2C-4318-930C-2283F5B74DA4}" uniqueName="6" name="IsStrong" queryTableFieldId="6"/>
     <tableColumn id="7" xr3:uid="{E2805626-3591-4BA3-83F6-12A977BCCD9B}" uniqueName="7" name="IsTourist" queryTableFieldId="7"/>
     <tableColumn id="8" xr3:uid="{4D5D6C14-27D9-4A98-AB67-29B05B62727D}" uniqueName="8" name="IsWeak" queryTableFieldId="8"/>
@@ -563,10 +572,10 @@
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.81640625" customWidth="1"/>
     <col min="3" max="3" width="8.81640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="8.1796875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.36328125" customWidth="1"/>
     <col min="6" max="6" width="9.90625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="10.26953125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="9.1796875" bestFit="1" customWidth="1"/>
@@ -587,94 +596,94 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
+        <v>20</v>
+      </c>
+      <c r="F1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>7</v>
-      </c>
-      <c r="I1" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A2" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C2" s="1" t="s">
+      <c r="A2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2">
+        <v>100</v>
+      </c>
+      <c r="F2">
+        <v>1</v>
+      </c>
+      <c r="G2">
+        <v>0</v>
+      </c>
+      <c r="H2">
+        <v>0</v>
+      </c>
+      <c r="I2" t="s">
         <v>11</v>
-      </c>
-      <c r="D2">
-        <v>1</v>
-      </c>
-      <c r="E2">
-        <v>0</v>
-      </c>
-      <c r="F2">
-        <v>1</v>
-      </c>
-      <c r="G2">
-        <v>0</v>
-      </c>
-      <c r="H2">
-        <v>0</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A3" s="1" t="s">
+      <c r="A3" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C3" t="s">
         <v>13</v>
       </c>
-      <c r="B3" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>11</v>
-      </c>
       <c r="D3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E3">
-        <v>0</v>
+        <v>95</v>
       </c>
       <c r="F3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H3">
         <v>0</v>
       </c>
-      <c r="I3" s="1" t="s">
-        <v>12</v>
+      <c r="I3" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A4" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>17</v>
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C4" t="s">
+        <v>13</v>
       </c>
       <c r="D4">
         <v>1</v>
       </c>
       <c r="E4">
-        <v>1</v>
+        <v>85</v>
       </c>
       <c r="F4">
         <v>1</v>
@@ -685,141 +694,141 @@
       <c r="H4">
         <v>0</v>
       </c>
-      <c r="I4" s="1" t="s">
-        <v>18</v>
+      <c r="I4" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A5" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>17</v>
+      <c r="A5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" t="s">
+        <v>24</v>
+      </c>
+      <c r="C5" t="s">
+        <v>9</v>
       </c>
       <c r="D5">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E5">
-        <v>1</v>
+        <v>60</v>
       </c>
       <c r="F5">
         <v>1</v>
       </c>
       <c r="G5">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H5">
         <v>0</v>
       </c>
-      <c r="I5" s="1" t="s">
-        <v>15</v>
+      <c r="I5" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A6" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>17</v>
+      <c r="A6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B6" t="s">
+        <v>25</v>
+      </c>
+      <c r="C6" t="s">
+        <v>13</v>
       </c>
       <c r="D6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E6">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="F6">
         <v>0</v>
       </c>
       <c r="G6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H6">
         <v>1</v>
       </c>
-      <c r="I6" s="1" t="s">
-        <v>12</v>
+      <c r="I6" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A7" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>17</v>
+      <c r="A7" t="s">
+        <v>16</v>
+      </c>
+      <c r="B7" t="s">
+        <v>26</v>
+      </c>
+      <c r="C7" t="s">
+        <v>9</v>
       </c>
       <c r="D7">
         <v>2</v>
       </c>
       <c r="E7">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="F7">
         <v>0</v>
       </c>
       <c r="G7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H7">
-        <v>0</v>
-      </c>
-      <c r="I7" s="1" t="s">
-        <v>12</v>
+        <v>1</v>
+      </c>
+      <c r="I7" t="s">
+        <v>10</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A8" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>26</v>
+      <c r="A8" t="s">
+        <v>17</v>
+      </c>
+      <c r="B8" t="s">
+        <v>27</v>
+      </c>
+      <c r="C8" t="s">
+        <v>18</v>
       </c>
       <c r="D8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E8">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="F8">
         <v>0</v>
       </c>
       <c r="G8">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H8">
         <v>0</v>
       </c>
-      <c r="I8" s="1" t="s">
-        <v>12</v>
+      <c r="I8" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A9" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="B9" s="1" t="s">
+      <c r="A9" t="s">
+        <v>19</v>
+      </c>
+      <c r="B9" t="s">
         <v>28</v>
       </c>
-      <c r="C9" s="1" t="s">
-        <v>26</v>
+      <c r="C9" t="s">
+        <v>18</v>
       </c>
       <c r="D9">
         <v>2</v>
       </c>
       <c r="E9">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="F9">
         <v>0</v>
@@ -828,10 +837,10 @@
         <v>0</v>
       </c>
       <c r="H9">
-        <v>1</v>
-      </c>
-      <c r="I9" s="1" t="s">
-        <v>12</v>
+        <v>0</v>
+      </c>
+      <c r="I9" t="s">
+        <v>17</v>
       </c>
     </row>
   </sheetData>

</xml_diff>